<commit_message>
fix(lib): fix Framework name for "Règles OIV - Secteur « Activités civiles de l'Etat »" (#3958)
Fix Framework Name
</commit_message>
<xml_diff>
--- a/tools/excel/lpm/lpm-oiv-2019_activites-civiles-de-l-etat.xlsx
+++ b/tools/excel/lpm/lpm-oiv-2019_activites-civiles-de-l-etat.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\tarkadia\projects\intuitem\ciso-assistant-community\tools\excel\lpm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96BB87C9-F30D-41D6-A430-5DC7DD56BFE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88C9CDBF-6FEE-4183-B257-525F4992B27D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="26448" yWindow="-10908" windowWidth="32208" windowHeight="16812" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3165" yWindow="-13275" windowWidth="15765" windowHeight="9870" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="library_meta" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="207">
   <si>
     <t>type</t>
   </si>
@@ -641,7 +641,10 @@
     <t>LPM-OIV-2019_Activites-civiles-de-l-etat</t>
   </si>
   <si>
-    <t>Règles OIV - Secteur « Activités civiles de l'Etat »</t>
+    <t>Règles OIV - Secteur « Activités civiles de l'Etat » (2019)</t>
+  </si>
+  <si>
+    <t>3</t>
   </si>
 </sst>
 </file>
@@ -794,43 +797,43 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -867,41 +870,6 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -1064,13 +1032,6 @@
       </border>
     </dxf>
     <dxf>
-      <border>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -1084,6 +1045,48 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
       </border>
     </dxf>
   </dxfs>
@@ -1102,13 +1105,13 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2B083513-3C40-42B8-8D00-7E62A104F6D5}" name="Tableau1" displayName="Tableau1" ref="A1:E182" totalsRowShown="0" headerRowDxfId="1" headerRowBorderDxfId="7" tableBorderDxfId="8" totalsRowBorderDxfId="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2B083513-3C40-42B8-8D00-7E62A104F6D5}" name="Tableau1" displayName="Tableau1" ref="A1:E182" totalsRowShown="0" headerRowDxfId="8" headerRowBorderDxfId="7" tableBorderDxfId="6" totalsRowBorderDxfId="5">
   <autoFilter ref="A1:E182" xr:uid="{2B083513-3C40-42B8-8D00-7E62A104F6D5}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{F12F13AA-41E2-4523-90A3-EFF6C41D17DF}" name="assessable" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{D376ED4D-D6AF-453F-81FD-FF3E6D0F45FD}" name="depth" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{220A56BB-42AC-4C5E-84AF-DC8AC2EC195C}" name="ref_id" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{BC85C096-5A43-4AEA-9390-63EA45670508}" name="name" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{F12F13AA-41E2-4523-90A3-EFF6C41D17DF}" name="assessable" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{D376ED4D-D6AF-453F-81FD-FF3E6D0F45FD}" name="depth" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{220A56BB-42AC-4C5E-84AF-DC8AC2EC195C}" name="ref_id" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{BC85C096-5A43-4AEA-9390-63EA45670508}" name="name" dataDxfId="1"/>
     <tableColumn id="5" xr3:uid="{DA60DCC1-3C56-4E31-86FB-AB7C50B6ACBB}" name="description" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="Style de tableau 1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1427,8 +1430,8 @@
       <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="2">
-        <v>2</v>
+      <c r="B3" s="2" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">

</xml_diff>